<commit_message>
Simplificar nombres de columnas en archivo tiendas_item
El archivo DB_Tiendas Por itmes y portafolio.xlsx ya no usa el prefijo
DB_Portafolio_Fruver. en sus columnas (ITEM, ESTADO, DESCRIPCION), por
lo que loader.py y preprocessor.py se actualizan para leerlas sin
prefijo. Se actualizan también los Input/*.xlsx con los datos más
recientes.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Input/Stock.xlsx
+++ b/Input/Stock.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prestamo\Documents\Isimo\Proyectos\Distribucion de Fruver\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8DB5B0C-8B9B-474F-8AD2-3C9901B2B2B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFDFA431-3884-47FF-8AF5-3CA579825046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="83">
   <si>
     <t>Item</t>
   </si>
@@ -116,151 +116,186 @@
     <t>001 - ACTIVO</t>
   </si>
   <si>
+    <t xml:space="preserve">FRUTAS FRESCAS                          </t>
+  </si>
+  <si>
+    <t>CN12</t>
+  </si>
+  <si>
+    <t>001 - REFRIGERADO</t>
+  </si>
+  <si>
+    <t>CN08</t>
+  </si>
+  <si>
+    <t>CN10</t>
+  </si>
+  <si>
+    <t>CN06</t>
+  </si>
+  <si>
+    <t>FRUTA IMPORTADA</t>
+  </si>
+  <si>
+    <t>AGUACATE HASS UND</t>
+  </si>
+  <si>
+    <t>CN36</t>
+  </si>
+  <si>
+    <t>CN25</t>
+  </si>
+  <si>
+    <t>MANZANA VERDE UND</t>
+  </si>
+  <si>
+    <t>KIWI 200 G</t>
+  </si>
+  <si>
+    <t>CN15</t>
+  </si>
+  <si>
+    <t>AGUACATE VARIEDAD UNIDAD</t>
+  </si>
+  <si>
+    <t>LIMON TAHITI 500 G</t>
+  </si>
+  <si>
+    <t>PLATANO UND</t>
+  </si>
+  <si>
+    <t>CN24</t>
+  </si>
+  <si>
+    <t>MANZANA ROYAL BOLSA  500 G</t>
+  </si>
+  <si>
+    <t>CN20</t>
+  </si>
+  <si>
+    <t>MANZANA MIXTA LONCHERA 500 G</t>
+  </si>
+  <si>
+    <t>ZANAHORIA 600 G</t>
+  </si>
+  <si>
+    <t>PAPAYA MEDIANA UNIDAD</t>
+  </si>
+  <si>
+    <t>PIMENTON 300 G</t>
+  </si>
+  <si>
+    <t>LULO 600 G</t>
+  </si>
+  <si>
+    <t>MANZANA  ROYAL GALA UND</t>
+  </si>
+  <si>
+    <t>PEPINO COHOMBRO UND</t>
+  </si>
+  <si>
+    <t>UVA VERDE SIN SEMILLA 400 G</t>
+  </si>
+  <si>
+    <t>UVA RED GLOBE 400 G</t>
+  </si>
+  <si>
+    <t>C100</t>
+  </si>
+  <si>
+    <t>BANANO UNIDAD</t>
+  </si>
+  <si>
+    <t>TOMATE  DE ARBOL 500 G</t>
+  </si>
+  <si>
+    <t>PINA UNIDAD</t>
+  </si>
+  <si>
+    <t>TOMATE CHONTO 500 G</t>
+  </si>
+  <si>
+    <t>PLATANO HARTON 1000 G</t>
+  </si>
+  <si>
     <t>ARANDANOS FRESCOS 125 G</t>
   </si>
   <si>
-    <t xml:space="preserve">FRUTAS FRESCAS                          </t>
-  </si>
-  <si>
-    <t>CN12</t>
-  </si>
-  <si>
-    <t>001 - REFRIGERADO</t>
+    <t>CN50</t>
+  </si>
+  <si>
+    <t>AJO 3 UND</t>
+  </si>
+  <si>
+    <t>002 - PROPIA</t>
+  </si>
+  <si>
+    <t>TOMATE CHERRY PURE VALLEY 250 G</t>
+  </si>
+  <si>
+    <t>MANZANA VERDE BOLSA  500 G</t>
+  </si>
+  <si>
+    <t>CEBOLLA LARGA 500G</t>
+  </si>
+  <si>
+    <t>MIX FRUTAS IMPORTADAS</t>
+  </si>
+  <si>
+    <t>PAPA PAREJA  1000 G</t>
+  </si>
+  <si>
+    <t>CN22</t>
+  </si>
+  <si>
+    <t>PERA VERDE IMPORTADA UNIDAD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">005 - PRODUCTO PRUEBA                         </t>
+  </si>
+  <si>
+    <t>CHAMPINON ENTERO 250 G</t>
+  </si>
+  <si>
+    <t>UVA ISABELA 400 G</t>
+  </si>
+  <si>
+    <t>SANDIA BABY UNIDAD</t>
+  </si>
+  <si>
+    <t>CIRUELA NACIONAL 400 G</t>
+  </si>
+  <si>
+    <t>BROCOLI 250 G</t>
+  </si>
+  <si>
+    <t>LECHUGA CRESPA VERDE  UNIDAD</t>
+  </si>
+  <si>
+    <t>ESPINACA  150 G</t>
+  </si>
+  <si>
+    <t>COGOLLO  3 UNIDADES 300 G</t>
+  </si>
+  <si>
+    <t>CEBOLLA ROJA 500 G</t>
+  </si>
+  <si>
+    <t>PAPA 2000 G</t>
   </si>
   <si>
     <t>CEBOLLA BLANCA CABEZONA 500 G</t>
-  </si>
-  <si>
-    <t>CN08</t>
-  </si>
-  <si>
-    <t>PLATANO HARTON 1000 G</t>
-  </si>
-  <si>
-    <t>CN10</t>
-  </si>
-  <si>
-    <t>CN06</t>
-  </si>
-  <si>
-    <t>ESPINACA  150 G</t>
-  </si>
-  <si>
-    <t>BANANO UNIDAD</t>
-  </si>
-  <si>
-    <t>C100</t>
-  </si>
-  <si>
-    <t>FRUTA IMPORTADA</t>
-  </si>
-  <si>
-    <t>AGUACATE HASS UND</t>
-  </si>
-  <si>
-    <t>CN36</t>
-  </si>
-  <si>
-    <t>CN25</t>
-  </si>
-  <si>
-    <t>MANZANA VERDE UND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">005 - PRODUCTO PRUEBA                         </t>
-  </si>
-  <si>
-    <t>GRANADILLA  450 G</t>
-  </si>
-  <si>
-    <t>MIX FRUTAS IMPORTADAS</t>
-  </si>
-  <si>
-    <t>ZANAHORIA 600 G</t>
-  </si>
-  <si>
-    <t>TOMATE CHERRY PURE VALLEY 250 G</t>
-  </si>
-  <si>
-    <t>002 - PROPIA</t>
-  </si>
-  <si>
-    <t>TOMATE CHONTO 500 G</t>
-  </si>
-  <si>
-    <t>TOMATE  DE ARBOL 500 G</t>
-  </si>
-  <si>
-    <t>UVA RED GLOBE 400 G</t>
-  </si>
-  <si>
-    <t>UVA VERDE SIN SEMILLA 400 G</t>
-  </si>
-  <si>
-    <t>SANDIA BABY UNIDAD</t>
-  </si>
-  <si>
-    <t>PAPAYA MEDIANA UNIDAD</t>
-  </si>
-  <si>
-    <t>LECHUGA BATAVIA UND</t>
-  </si>
-  <si>
-    <t>CJ10</t>
-  </si>
-  <si>
-    <t>FLOR DE JAMAICA 15 G</t>
-  </si>
-  <si>
-    <t>RAIZ CHINA 150 G</t>
-  </si>
-  <si>
-    <t>LULO 600 G</t>
-  </si>
-  <si>
-    <t>LECHUGA CRESPA VERDE  UNIDAD</t>
-  </si>
-  <si>
-    <t>PIMENTON 300 G</t>
-  </si>
-  <si>
-    <t>NARANJA TANGELO 1000 G</t>
-  </si>
-  <si>
-    <t>KIWI 200 G</t>
-  </si>
-  <si>
-    <t>BROCOLI 250 G</t>
-  </si>
-  <si>
-    <t>PEPINO COHOMBRO UND</t>
-  </si>
-  <si>
-    <t>CN15</t>
-  </si>
-  <si>
-    <t>AGUACATE VARIEDAD UNIDAD</t>
-  </si>
-  <si>
-    <t>LIMON TAHITI 500 G</t>
-  </si>
-  <si>
-    <t>PURE VALLEY</t>
-  </si>
-  <si>
-    <t>NO APLICA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="##,##0.0000"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="##,##0.00"/>
     <numFmt numFmtId="167" formatCode="0000000"/>
-    <numFmt numFmtId="168" formatCode="d\/mm\/yyyy"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -300,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -336,12 +371,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -665,7 +694,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:R30"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="13.5703125" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="8.5703125" customWidth="1"/>
@@ -687,7 +716,7 @@
     <col min="17" max="17" width="19.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -740,102 +769,98 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="12">
+        <v>155</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="11">
+        <v>18</v>
+      </c>
+      <c r="H2" s="11">
+        <v>10</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="N2" s="10">
+        <v>861499.48</v>
+      </c>
+      <c r="O2" s="9">
+        <v>50</v>
+      </c>
+      <c r="P2" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="7">
         <v>157</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="8" t="s">
+      <c r="E3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="6">
+        <v>3</v>
+      </c>
+      <c r="H3" s="6">
+        <v>1</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2" s="11">
-        <v>3</v>
-      </c>
-      <c r="H2" s="11">
-        <v>3</v>
-      </c>
-      <c r="I2" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L2" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="M2" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="N2" s="10">
-        <v>232485.47</v>
-      </c>
-      <c r="O2" s="9">
-        <v>12</v>
-      </c>
-      <c r="P2" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="13">
-        <v>46182</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="7">
-        <v>175</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="6">
-        <v>13</v>
-      </c>
-      <c r="H3" s="6">
-        <v>10</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>23</v>
-      </c>
       <c r="M3" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N3" s="5">
-        <v>360345.46</v>
+        <v>238458.95</v>
       </c>
       <c r="O3" s="4">
         <v>12</v>
@@ -843,17 +868,13 @@
       <c r="P3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="14">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="4" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="12">
-        <v>233</v>
+        <v>175</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>32</v>
+        <v>82</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>17</v>
@@ -862,16 +883,16 @@
         <v>18</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>19</v>
       </c>
       <c r="G4" s="11">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="H4" s="11">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="I4" s="8" t="s">
         <v>20</v>
@@ -889,7 +910,7 @@
         <v>24</v>
       </c>
       <c r="N4" s="10">
-        <v>913333.76000000001</v>
+        <v>1242443.8600000001</v>
       </c>
       <c r="O4" s="9">
         <v>12</v>
@@ -897,17 +918,13 @@
       <c r="P4" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="Q4" s="8"/>
-      <c r="R4" s="13">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="5" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="7">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>49</v>
+        <v>81</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>17</v>
@@ -916,16 +933,16 @@
         <v>18</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G5" s="6">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="H5" s="6">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="I5" s="3" t="s">
         <v>20</v>
@@ -943,25 +960,21 @@
         <v>24</v>
       </c>
       <c r="N5" s="5">
-        <v>1529982.87</v>
+        <v>1252434.52</v>
       </c>
       <c r="O5" s="4">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="P5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="14">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="6" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="12">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>17</v>
@@ -970,16 +983,16 @@
         <v>18</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>19</v>
       </c>
       <c r="G6" s="11">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="H6" s="11">
-        <v>5</v>
+        <v>51</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>20</v>
@@ -997,43 +1010,39 @@
         <v>24</v>
       </c>
       <c r="N6" s="10">
-        <v>295627.27</v>
+        <v>2359372.52</v>
       </c>
       <c r="O6" s="9">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="P6" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="Q6" s="8"/>
-      <c r="R6" s="13">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="7" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="7">
-        <v>965</v>
+        <v>235</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G7" s="6">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="H7" s="6">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="I7" s="3" t="s">
         <v>20</v>
@@ -1051,25 +1060,21 @@
         <v>24</v>
       </c>
       <c r="N7" s="5">
-        <v>1271907.95</v>
+        <v>2550550.0699999998</v>
       </c>
       <c r="O7" s="4">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="P7" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="14">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="8" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="12">
-        <v>1072</v>
+        <v>238</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>17</v>
@@ -1078,16 +1083,16 @@
         <v>18</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>19</v>
       </c>
       <c r="G8" s="11">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="H8" s="11">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>20</v>
@@ -1099,13 +1104,13 @@
         <v>22</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M8" s="8" t="s">
         <v>24</v>
       </c>
       <c r="N8" s="10">
-        <v>357704.99</v>
+        <v>527580.47</v>
       </c>
       <c r="O8" s="9">
         <v>10</v>
@@ -1113,35 +1118,31 @@
       <c r="P8" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="Q8" s="8"/>
-      <c r="R8" s="13">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="9" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="7">
-        <v>1074</v>
+        <v>754</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>66</v>
-      </c>
       <c r="F9" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G9" s="6">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="H9" s="6">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>20</v>
@@ -1159,43 +1160,39 @@
         <v>24</v>
       </c>
       <c r="N9" s="5">
-        <v>3238894.04</v>
+        <v>178091.96</v>
       </c>
       <c r="O9" s="4">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="P9" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="14">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="10" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="12">
-        <v>1079</v>
+        <v>883</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>17</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>19</v>
       </c>
       <c r="G10" s="11">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="H10" s="11">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I10" s="8" t="s">
         <v>20</v>
@@ -1207,49 +1204,45 @@
         <v>22</v>
       </c>
       <c r="L10" s="8" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M10" s="8" t="s">
         <v>24</v>
       </c>
       <c r="N10" s="10">
-        <v>185372.51</v>
+        <v>369168.64000000001</v>
       </c>
       <c r="O10" s="9">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="P10" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="Q10" s="8"/>
-      <c r="R10" s="13">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="11" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="7">
-        <v>1156</v>
+        <v>965</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>33</v>
-      </c>
       <c r="F11" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G11" s="6">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="H11" s="6">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>20</v>
@@ -1267,97 +1260,89 @@
         <v>24</v>
       </c>
       <c r="N11" s="5">
-        <v>298112.62</v>
+        <v>856426.55</v>
       </c>
       <c r="O11" s="4">
+        <v>12</v>
+      </c>
+      <c r="P11" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A12" s="12">
+        <v>1071</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G12" s="11">
+        <v>5</v>
+      </c>
+      <c r="H12" s="11">
+        <v>5</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L12" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="M12" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="N12" s="10">
+        <v>296251.23</v>
+      </c>
+      <c r="O12" s="9">
         <v>10</v>
       </c>
-      <c r="P11" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q11" s="3"/>
-      <c r="R11" s="14">
-        <v>46183</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="12">
-        <v>1210</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G12" s="11">
-        <v>163</v>
-      </c>
-      <c r="H12" s="11">
-        <v>100</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K12" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L12" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="M12" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="N12" s="10">
-        <v>6214439.46</v>
-      </c>
-      <c r="O12" s="9">
-        <v>100</v>
-      </c>
       <c r="P12" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="13">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="13" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="7">
-        <v>1510</v>
+        <v>1072</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G13" s="6">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="H13" s="6">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="I13" s="3" t="s">
         <v>20</v>
@@ -1369,28 +1354,24 @@
         <v>22</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="M13" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N13" s="5">
-        <v>464317.15</v>
+        <v>565333.79</v>
       </c>
       <c r="O13" s="4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="P13" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Q13" s="3"/>
-      <c r="R13" s="14">
-        <v>46183</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="14" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="12">
-        <v>1561</v>
+        <v>1074</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>39</v>
@@ -1399,19 +1380,19 @@
         <v>17</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>19</v>
       </c>
       <c r="G14" s="11">
-        <v>142</v>
+        <v>35</v>
       </c>
       <c r="H14" s="11">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="I14" s="8" t="s">
         <v>20</v>
@@ -1429,43 +1410,39 @@
         <v>24</v>
       </c>
       <c r="N14" s="10">
-        <v>5110454.42</v>
+        <v>3344962.94</v>
       </c>
       <c r="O14" s="9">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="P14" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="Q14" s="8"/>
-      <c r="R14" s="13">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="15" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="7">
-        <v>1562</v>
+        <v>1079</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>52</v>
+        <v>77</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G15" s="6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H15" s="6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>20</v>
@@ -1477,49 +1454,45 @@
         <v>22</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="M15" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N15" s="5">
-        <v>742942.11</v>
+        <v>89281.31</v>
       </c>
       <c r="O15" s="4">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="P15" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="14">
-        <v>46183</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="16" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="12">
-        <v>1623</v>
+        <v>1156</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>17</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>19</v>
       </c>
       <c r="G16" s="11">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H16" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I16" s="8" t="s">
         <v>20</v>
@@ -1537,7 +1510,7 @@
         <v>24</v>
       </c>
       <c r="N16" s="10">
-        <v>164141.1</v>
+        <v>348924.25</v>
       </c>
       <c r="O16" s="9">
         <v>10</v>
@@ -1545,35 +1518,31 @@
       <c r="P16" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="Q16" s="8"/>
-      <c r="R16" s="13">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="17" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="17" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="7">
-        <v>1673</v>
+        <v>1210</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G17" s="6">
-        <v>5</v>
+        <v>149</v>
       </c>
       <c r="H17" s="6">
-        <v>5</v>
+        <v>101</v>
       </c>
       <c r="I17" s="3" t="s">
         <v>20</v>
@@ -1591,99 +1560,89 @@
         <v>24</v>
       </c>
       <c r="N17" s="5">
-        <v>204642.2</v>
+        <v>5683445.46</v>
       </c>
       <c r="O17" s="4">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="P17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Q17" s="3"/>
-      <c r="R17" s="14">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="18" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="12">
-        <v>1795</v>
+        <v>1510</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>17</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E18" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G18" s="11">
+        <v>23</v>
+      </c>
+      <c r="H18" s="11">
+        <v>20</v>
+      </c>
+      <c r="I18" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J18" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K18" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L18" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="M18" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="N18" s="10">
+        <v>1557238.83</v>
+      </c>
+      <c r="O18" s="9">
+        <v>8</v>
+      </c>
+      <c r="P18" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="7">
+        <v>1561</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E19" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="F18" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G18" s="11">
-        <v>19</v>
-      </c>
-      <c r="H18" s="11">
-        <v>10</v>
-      </c>
-      <c r="I18" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J18" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K18" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L18" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="M18" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="N18" s="10">
-        <v>507250.62</v>
-      </c>
-      <c r="O18" s="9">
-        <v>6</v>
-      </c>
-      <c r="P18" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q18" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="R18" s="13">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="7">
-        <v>1800</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="F19" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G19" s="6">
-        <v>17</v>
+        <v>103</v>
       </c>
       <c r="H19" s="6">
-        <v>10</v>
+        <v>81</v>
       </c>
       <c r="I19" s="3" t="s">
         <v>20</v>
@@ -1701,43 +1660,39 @@
         <v>24</v>
       </c>
       <c r="N19" s="5">
-        <v>594020.05000000005</v>
+        <v>3580786.7</v>
       </c>
       <c r="O19" s="4">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="P19" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Q19" s="3"/>
-      <c r="R19" s="14">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="20" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="20" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="12">
-        <v>1803</v>
+        <v>1562</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>17</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>19</v>
       </c>
       <c r="G20" s="11">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="H20" s="11">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I20" s="8" t="s">
         <v>20</v>
@@ -1749,13 +1704,13 @@
         <v>22</v>
       </c>
       <c r="L20" s="8" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M20" s="8" t="s">
         <v>24</v>
       </c>
       <c r="N20" s="10">
-        <v>1219603.97</v>
+        <v>2019767.55</v>
       </c>
       <c r="O20" s="9">
         <v>8</v>
@@ -1763,35 +1718,31 @@
       <c r="P20" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="Q20" s="8"/>
-      <c r="R20" s="13">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="21" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="21" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="7">
-        <v>1804</v>
+        <v>1601</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D21" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G21" s="6">
         <v>27</v>
       </c>
-      <c r="E21" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G21" s="6">
-        <v>3</v>
-      </c>
       <c r="H21" s="6">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="I21" s="3" t="s">
         <v>20</v>
@@ -1803,49 +1754,45 @@
         <v>22</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N21" s="5">
-        <v>125617.57</v>
+        <v>1556070.51</v>
       </c>
       <c r="O21" s="4">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="P21" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Q21" s="3"/>
-      <c r="R21" s="14">
-        <v>46182</v>
-      </c>
-    </row>
-    <row r="22" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="22" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="12">
-        <v>1806</v>
+        <v>1623</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>17</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>19</v>
       </c>
       <c r="G22" s="11">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H22" s="11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>20</v>
@@ -1863,43 +1810,39 @@
         <v>24</v>
       </c>
       <c r="N22" s="10">
-        <v>338548.08</v>
+        <v>173232.4</v>
       </c>
       <c r="O22" s="9">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="P22" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="Q22" s="8"/>
-      <c r="R22" s="13">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="23" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="23" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="7">
-        <v>1812</v>
+        <v>1671</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G23" s="6">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="H23" s="6">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="I23" s="3" t="s">
         <v>20</v>
@@ -1917,43 +1860,39 @@
         <v>24</v>
       </c>
       <c r="N23" s="5">
-        <v>688319.92</v>
+        <v>1210803.23</v>
       </c>
       <c r="O23" s="4">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="P23" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Q23" s="3"/>
-      <c r="R23" s="14">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="24" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="24" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="12">
-        <v>1822</v>
+        <v>1673</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>17</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>19</v>
       </c>
       <c r="G24" s="11">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="H24" s="11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I24" s="8" t="s">
         <v>20</v>
@@ -1965,33 +1904,27 @@
         <v>22</v>
       </c>
       <c r="L24" s="8" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="M24" s="8" t="s">
         <v>24</v>
       </c>
       <c r="N24" s="10">
-        <v>152432.28</v>
+        <v>591858.44999999995</v>
       </c>
       <c r="O24" s="9">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="P24" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q24" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="R24" s="13">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="25" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="7">
-        <v>2001</v>
+        <v>1795</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>17</v>
@@ -2000,88 +1933,84 @@
         <v>18</v>
       </c>
       <c r="E25" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G25" s="6">
+        <v>10</v>
+      </c>
+      <c r="H25" s="6">
+        <v>10</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L25" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F25" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G25" s="6">
-        <v>9</v>
-      </c>
-      <c r="H25" s="6">
-        <v>5</v>
-      </c>
-      <c r="I25" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J25" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K25" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="L25" s="3" t="s">
+      <c r="M25" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="N25" s="5">
+        <v>277726.56</v>
+      </c>
+      <c r="O25" s="4">
+        <v>6</v>
+      </c>
+      <c r="P25" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="12">
+        <v>1797</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G26" s="11">
+        <v>10</v>
+      </c>
+      <c r="H26" s="11">
+        <v>10</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J26" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K26" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L26" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="M25" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="N25" s="5">
-        <v>106017.59</v>
-      </c>
-      <c r="O25" s="4">
-        <v>12</v>
-      </c>
-      <c r="P25" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q25" s="3"/>
-      <c r="R25" s="14">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="26" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="12">
-        <v>2050</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G26" s="11">
-        <v>5</v>
-      </c>
-      <c r="H26" s="11">
-        <v>5</v>
-      </c>
-      <c r="I26" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J26" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K26" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L26" s="8" t="s">
-        <v>29</v>
-      </c>
       <c r="M26" s="8" t="s">
         <v>24</v>
       </c>
       <c r="N26" s="10">
-        <v>256261.12</v>
+        <v>176669.1</v>
       </c>
       <c r="O26" s="9">
         <v>6</v>
@@ -2089,35 +2018,31 @@
       <c r="P26" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="Q26" s="8"/>
-      <c r="R26" s="13">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="27" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="27" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="7">
-        <v>2473</v>
+        <v>1803</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>17</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>19</v>
       </c>
       <c r="G27" s="6">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="H27" s="6">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>20</v>
@@ -2129,13 +2054,13 @@
         <v>22</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="M27" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N27" s="5">
-        <v>796631.23</v>
+        <v>767050.21</v>
       </c>
       <c r="O27" s="4">
         <v>8</v>
@@ -2143,173 +2068,705 @@
       <c r="P27" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="Q27" s="3"/>
-      <c r="R27" s="14">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="28" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+    </row>
+    <row r="28" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="12">
+        <v>1804</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" s="11">
+        <v>5</v>
+      </c>
+      <c r="H28" s="11">
+        <v>4</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K28" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L28" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="M28" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="N28" s="10">
+        <v>205622.21</v>
+      </c>
+      <c r="O28" s="9">
+        <v>8</v>
+      </c>
+      <c r="P28" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A29" s="7">
+        <v>1808</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G29" s="6">
+        <v>12</v>
+      </c>
+      <c r="H29" s="6">
+        <v>10</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L29" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="M29" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="N29" s="5">
+        <v>676087.14</v>
+      </c>
+      <c r="O29" s="4">
+        <v>12</v>
+      </c>
+      <c r="P29" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A30" s="12">
+        <v>1812</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G30" s="11">
+        <v>3</v>
+      </c>
+      <c r="H30" s="11">
+        <v>3</v>
+      </c>
+      <c r="I30" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K30" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L30" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="M30" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="N30" s="10">
+        <v>129722.96</v>
+      </c>
+      <c r="O30" s="9">
+        <v>8</v>
+      </c>
+      <c r="P30" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="7">
+        <v>1813</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G31" s="6">
+        <v>20</v>
+      </c>
+      <c r="H31" s="6">
+        <v>20</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K31" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L31" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M31" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="N31" s="5">
+        <v>370400.34</v>
+      </c>
+      <c r="O31" s="4">
+        <v>6</v>
+      </c>
+      <c r="P31" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A32" s="12">
+        <v>1815</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G32" s="11">
+        <v>30</v>
+      </c>
+      <c r="H32" s="11">
+        <v>30</v>
+      </c>
+      <c r="I32" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J32" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K32" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L32" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="M32" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="N32" s="10">
+        <v>2010000</v>
+      </c>
+      <c r="O32" s="9">
+        <v>10</v>
+      </c>
+      <c r="P32" s="8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A33" s="7">
+        <v>1867</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G33" s="6">
+        <v>40</v>
+      </c>
+      <c r="H33" s="6">
+        <v>40</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J33" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K33" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L33" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="M33" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="N33" s="5">
+        <v>969893.44</v>
+      </c>
+      <c r="O33" s="4">
+        <v>22</v>
+      </c>
+      <c r="P33" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A34" s="12">
+        <v>1868</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G34" s="11">
+        <v>10</v>
+      </c>
+      <c r="H34" s="11">
+        <v>10</v>
+      </c>
+      <c r="I34" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J34" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K34" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L34" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="M34" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="N34" s="10">
+        <v>320866.24</v>
+      </c>
+      <c r="O34" s="9">
+        <v>10</v>
+      </c>
+      <c r="P34" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A35" s="7">
+        <v>2001</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G35" s="6">
+        <v>19</v>
+      </c>
+      <c r="H35" s="6">
+        <v>15</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K35" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L35" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M35" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="N35" s="5">
+        <v>273613.43</v>
+      </c>
+      <c r="O35" s="4">
+        <v>12</v>
+      </c>
+      <c r="P35" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A36" s="12">
+        <v>2050</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G36" s="11">
+        <v>10</v>
+      </c>
+      <c r="H36" s="11">
+        <v>10</v>
+      </c>
+      <c r="I36" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J36" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K36" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L36" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="M36" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="N36" s="10">
+        <v>466511.14</v>
+      </c>
+      <c r="O36" s="9">
+        <v>6</v>
+      </c>
+      <c r="P36" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A37" s="7">
+        <v>2052</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G37" s="6">
+        <v>10</v>
+      </c>
+      <c r="H37" s="6">
+        <v>10</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J37" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K37" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L37" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="M37" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="N37" s="5">
+        <v>346613.81</v>
+      </c>
+      <c r="O37" s="4">
+        <v>10</v>
+      </c>
+      <c r="P37" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A38" s="12">
+        <v>2243</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G38" s="11">
+        <v>25</v>
+      </c>
+      <c r="H38" s="11">
+        <v>25</v>
+      </c>
+      <c r="I38" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J38" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K38" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L38" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="M38" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="N38" s="10">
+        <v>2126591.92</v>
+      </c>
+      <c r="O38" s="9">
+        <v>20</v>
+      </c>
+      <c r="P38" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A39" s="7">
+        <v>2244</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G39" s="6">
+        <v>20</v>
+      </c>
+      <c r="H39" s="6">
+        <v>20</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K39" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L39" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="M39" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="N39" s="5">
+        <v>1941218.17</v>
+      </c>
+      <c r="O39" s="4">
+        <v>20</v>
+      </c>
+      <c r="P39" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A40" s="12">
+        <v>2473</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G40" s="11">
+        <v>24</v>
+      </c>
+      <c r="H40" s="11">
+        <v>20</v>
+      </c>
+      <c r="I40" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="J40" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K40" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="L40" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="M40" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="N40" s="10">
+        <v>754597.79</v>
+      </c>
+      <c r="O40" s="9">
+        <v>8</v>
+      </c>
+      <c r="P40" s="8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A41" s="7">
         <v>2604</v>
       </c>
-      <c r="B28" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D28" s="8" t="s">
+      <c r="B41" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E41" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E28" s="8" t="s">
+      <c r="F41" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G41" s="6">
+        <v>15</v>
+      </c>
+      <c r="H41" s="6">
+        <v>15</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K41" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L41" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F28" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G28" s="11">
-        <v>16</v>
-      </c>
-      <c r="H28" s="11">
-        <v>5</v>
-      </c>
-      <c r="I28" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J28" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K28" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L28" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="M28" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="N28" s="10">
-        <v>580180.35</v>
-      </c>
-      <c r="O28" s="9">
+      <c r="M41" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="N41" s="5">
+        <v>544180.35</v>
+      </c>
+      <c r="O41" s="4">
         <v>12</v>
       </c>
-      <c r="P28" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q28" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="R28" s="13">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="29" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="7">
-        <v>3100</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G29" s="6">
-        <v>1</v>
-      </c>
-      <c r="H29" s="6">
-        <v>1</v>
-      </c>
-      <c r="I29" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K29" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="L29" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M29" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="N29" s="5">
-        <v>20569.099999999999</v>
-      </c>
-      <c r="O29" s="4">
-        <v>10</v>
-      </c>
-      <c r="P29" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q29" s="3"/>
-      <c r="R29" s="14">
-        <v>46184</v>
-      </c>
-    </row>
-    <row r="30" spans="1:18" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="12">
-        <v>3112</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D30" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="F30" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G30" s="11">
-        <v>14</v>
-      </c>
-      <c r="H30" s="11">
-        <v>10</v>
-      </c>
-      <c r="I30" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="J30" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K30" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L30" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="M30" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="N30" s="10">
-        <v>396237.84</v>
-      </c>
-      <c r="O30" s="9">
-        <v>10</v>
-      </c>
-      <c r="P30" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q30" s="8"/>
-      <c r="R30" s="13">
-        <v>46184</v>
+      <c r="P41" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>